<commit_message>
Add lab6_1 for JunitTest and Update template_Lab6.xlsx
</commit_message>
<xml_diff>
--- a/Lab06/Test_Cases/template_Lab6.xlsx
+++ b/Lab06/Test_Cases/template_Lab6.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ThirdYearTerm1\Sqa\Lab06\Test_Cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDF60F82-C63A-4F0D-8585-4F62963DE454}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA13CCB3-75A6-4489-B692-F6BF12A60FAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4365" yWindow="2565" windowWidth="21600" windowHeight="11835" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3600" yWindow="2475" windowWidth="21600" windowHeight="11835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Limited Entry Decision Table" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="74">
   <si>
     <t>Condition</t>
   </si>
@@ -258,6 +258,9 @@
   </si>
   <si>
     <t>REAL_ROOTS</t>
+  </si>
+  <si>
+    <t>Pass</t>
   </si>
 </sst>
 </file>
@@ -515,6 +518,8 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -536,8 +541,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -56917,15 +56920,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="29"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="31"/>
     </row>
     <row r="2" spans="1:8" ht="15.75" customHeight="1">
       <c r="A2" s="6"/>
@@ -56940,12 +56943,12 @@
       <c r="A3" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="28"/>
-      <c r="D3" s="28"/>
-      <c r="E3" s="28"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
       <c r="F3" s="12" t="s">
         <v>13</v>
       </c>
@@ -56957,12 +56960,12 @@
       <c r="A4" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="30" t="s">
+      <c r="B4" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="28"/>
-      <c r="D4" s="28"/>
-      <c r="E4" s="28"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
       <c r="F4" s="12" t="s">
         <v>19</v>
       </c>
@@ -56974,10 +56977,10 @@
       <c r="A5" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="31"/>
-      <c r="C5" s="28"/>
-      <c r="D5" s="28"/>
-      <c r="E5" s="29"/>
+      <c r="B5" s="33"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="31"/>
       <c r="F5" s="12" t="s">
         <v>24</v>
       </c>
@@ -56995,30 +56998,30 @@
       <c r="G6" s="7"/>
     </row>
     <row r="7" spans="1:8" ht="27" customHeight="1">
-      <c r="A7" s="32" t="s">
+      <c r="A7" s="34" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="24" t="s">
+      <c r="B7" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="31" t="s">
+      <c r="C7" s="33" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="28"/>
-      <c r="E7" s="29"/>
-      <c r="F7" s="24" t="s">
+      <c r="D7" s="30"/>
+      <c r="E7" s="31"/>
+      <c r="F7" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="G7" s="24" t="s">
+      <c r="G7" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="H7" s="26" t="s">
+      <c r="H7" s="28" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A8" s="25"/>
-      <c r="B8" s="25"/>
+      <c r="A8" s="27"/>
+      <c r="B8" s="27"/>
       <c r="C8" s="16" t="s">
         <v>34</v>
       </c>
@@ -57028,9 +57031,9 @@
       <c r="E8" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="F8" s="25"/>
-      <c r="G8" s="25"/>
-      <c r="H8" s="25"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="27"/>
     </row>
     <row r="9" spans="1:8" ht="15.75" customHeight="1">
       <c r="A9" s="17" t="str">
@@ -57049,11 +57052,15 @@
       <c r="E9" s="13">
         <v>6</v>
       </c>
-      <c r="F9" s="34" t="s">
+      <c r="F9" s="25" t="s">
         <v>72</v>
       </c>
-      <c r="G9" s="13"/>
-      <c r="H9" s="13"/>
+      <c r="G9" s="25" t="s">
+        <v>72</v>
+      </c>
+      <c r="H9" s="13" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="10" spans="1:8" ht="15.75" customHeight="1">
       <c r="A10" s="17" t="str">
@@ -57072,11 +57079,15 @@
       <c r="E10" s="13">
         <v>1</v>
       </c>
-      <c r="F10" s="34" t="s">
+      <c r="F10" s="25" t="s">
         <v>71</v>
       </c>
-      <c r="G10" s="13"/>
-      <c r="H10" s="13"/>
+      <c r="G10" s="25" t="s">
+        <v>71</v>
+      </c>
+      <c r="H10" s="13" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="11" spans="1:8" ht="15.75" customHeight="1">
       <c r="A11" s="17" t="str">
@@ -57095,11 +57106,15 @@
       <c r="E11" s="13">
         <v>1</v>
       </c>
-      <c r="F11" s="34" t="s">
+      <c r="F11" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="G11" s="13"/>
-      <c r="H11" s="13"/>
+      <c r="G11" s="25" t="s">
+        <v>70</v>
+      </c>
+      <c r="H11" s="13" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="12" spans="1:8" ht="15.75" customHeight="1">
       <c r="A12" s="17" t="str">
@@ -57118,11 +57133,15 @@
       <c r="E12" s="13">
         <v>1</v>
       </c>
-      <c r="F12" s="33" t="s">
+      <c r="F12" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="G12" s="13"/>
-      <c r="H12" s="13"/>
+      <c r="G12" s="24" t="s">
+        <v>69</v>
+      </c>
+      <c r="H12" s="13" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="13" spans="1:8" ht="15.75" customHeight="1">
       <c r="A13" s="19"/>
@@ -60196,15 +60215,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="29"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="31"/>
     </row>
     <row r="2" spans="1:8" ht="15.75" customHeight="1">
       <c r="A2" s="6"/>
@@ -60219,12 +60238,12 @@
       <c r="A3" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="28"/>
-      <c r="D3" s="28"/>
-      <c r="E3" s="28"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
       <c r="F3" s="12" t="s">
         <v>13</v>
       </c>
@@ -60236,12 +60255,12 @@
       <c r="A4" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="30" t="s">
+      <c r="B4" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="28"/>
-      <c r="D4" s="28"/>
-      <c r="E4" s="28"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
       <c r="F4" s="12" t="s">
         <v>19</v>
       </c>
@@ -60253,10 +60272,10 @@
       <c r="A5" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="31"/>
-      <c r="C5" s="28"/>
-      <c r="D5" s="28"/>
-      <c r="E5" s="29"/>
+      <c r="B5" s="33"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="31"/>
       <c r="F5" s="12" t="s">
         <v>24</v>
       </c>
@@ -60274,36 +60293,36 @@
       <c r="G6" s="7"/>
     </row>
     <row r="7" spans="1:8" ht="55.5" customHeight="1">
-      <c r="A7" s="32" t="s">
+      <c r="A7" s="34" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="24" t="s">
+      <c r="B7" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="31" t="s">
+      <c r="C7" s="33" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="28"/>
-      <c r="E7" s="29"/>
-      <c r="F7" s="24" t="s">
+      <c r="D7" s="30"/>
+      <c r="E7" s="31"/>
+      <c r="F7" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="G7" s="24" t="s">
+      <c r="G7" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="H7" s="26" t="s">
+      <c r="H7" s="28" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A8" s="25"/>
-      <c r="B8" s="25"/>
+      <c r="A8" s="27"/>
+      <c r="B8" s="27"/>
       <c r="C8" s="16"/>
       <c r="D8" s="16"/>
       <c r="E8" s="16"/>
-      <c r="F8" s="25"/>
-      <c r="G8" s="25"/>
-      <c r="H8" s="25"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="27"/>
     </row>
     <row r="9" spans="1:8" ht="15.75" customHeight="1">
       <c r="A9" s="17"/>

</xml_diff>

<commit_message>
Update template_Lab6 for Extended Entry DT
</commit_message>
<xml_diff>
--- a/Lab06/Test_Cases/template_Lab6.xlsx
+++ b/Lab06/Test_Cases/template_Lab6.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ThirdYearTerm1\Sqa\Lab06\Test_Cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA13CCB3-75A6-4489-B692-F6BF12A60FAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FDD2320-BBDA-4B6C-B5EF-704382D1197A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3600" yWindow="2475" windowWidth="21600" windowHeight="11835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Limited Entry Decision Table" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="63">
   <si>
     <t>Condition</t>
   </si>
@@ -63,9 +63,6 @@
   </si>
   <si>
     <t xml:space="preserve">Project Name: </t>
-  </si>
-  <si>
-    <t>EC1 =</t>
   </si>
   <si>
     <t>Lab 6.1</t>
@@ -99,9 +96,6 @@
   </si>
   <si>
     <t xml:space="preserve">Designer: </t>
-  </si>
-  <si>
-    <t>EC2 =</t>
   </si>
   <si>
     <t>นายกานดิทัต นามสุดตา</t>
@@ -173,79 +167,16 @@
     <t>TC004</t>
   </si>
   <si>
-    <t>Rule#5</t>
-  </si>
-  <si>
     <t>Not a quadratic equation</t>
-  </si>
-  <si>
-    <t>Rule#6</t>
-  </si>
-  <si>
-    <t>Rule#7</t>
-  </si>
-  <si>
-    <t>Rule#8</t>
   </si>
   <si>
     <t>Action</t>
   </si>
   <si>
-    <t>Rule#9</t>
-  </si>
-  <si>
-    <t>Rule#10</t>
-  </si>
-  <si>
-    <t>Rule#11</t>
-  </si>
-  <si>
-    <t>Rule#12</t>
-  </si>
-  <si>
-    <t>Rule#13</t>
-  </si>
-  <si>
-    <t>Rule#14</t>
-  </si>
-  <si>
-    <t>Rule#15</t>
-  </si>
-  <si>
-    <t>Rule#16</t>
-  </si>
-  <si>
-    <t>TC005</t>
-  </si>
-  <si>
     <t>X</t>
   </si>
   <si>
-    <t>TC006</t>
-  </si>
-  <si>
-    <t>TC007</t>
-  </si>
-  <si>
-    <t>TC008</t>
-  </si>
-  <si>
-    <t>TC009</t>
-  </si>
-  <si>
-    <t>TC010</t>
-  </si>
-  <si>
-    <t>TC011</t>
-  </si>
-  <si>
     <t>Impossible</t>
-  </si>
-  <si>
-    <t>TC012</t>
-  </si>
-  <si>
-    <t>TC013</t>
   </si>
   <si>
     <t>NOT_QUADRATIC</t>
@@ -261,6 +192,42 @@
   </si>
   <si>
     <t>Pass</t>
+  </si>
+  <si>
+    <t>EC1</t>
+  </si>
+  <si>
+    <t>EC2</t>
+  </si>
+  <si>
+    <t>EC3</t>
+  </si>
+  <si>
+    <t>EC4</t>
+  </si>
+  <si>
+    <t>EC5</t>
+  </si>
+  <si>
+    <t>EC1 = b² - 4ac &gt; 0</t>
+  </si>
+  <si>
+    <t>EC2 = b² - 4ac = 0</t>
+  </si>
+  <si>
+    <t>EC3 = b² - 4ac &lt; 0</t>
+  </si>
+  <si>
+    <t>EC4 = a = 0</t>
+  </si>
+  <si>
+    <t>EC5 = a ≠ 0   (a in range 1 - 100)</t>
+  </si>
+  <si>
+    <t>Value of a</t>
+  </si>
+  <si>
+    <t>Discriminant Value (b² - 4ac)</t>
   </si>
 </sst>
 </file>
@@ -362,7 +329,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -459,11 +426,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -515,11 +497,16 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -804,19 +791,19 @@
     </row>
     <row r="2" spans="1:26" ht="21" customHeight="1">
       <c r="A2" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="C2" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="11" t="s">
-        <v>12</v>
-      </c>
       <c r="D2" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F2" s="5"/>
       <c r="G2" s="5"/>
@@ -842,19 +829,19 @@
     </row>
     <row r="3" spans="1:26" ht="21" customHeight="1">
       <c r="A3" s="10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C3" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="11" t="s">
-        <v>12</v>
-      </c>
       <c r="E3" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="5"/>
@@ -869,7 +856,7 @@
       <c r="P3" s="5"/>
       <c r="Q3" s="4"/>
       <c r="R3" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S3" s="4"/>
       <c r="T3" s="4"/>
@@ -882,19 +869,19 @@
     </row>
     <row r="4" spans="1:26" ht="21" customHeight="1">
       <c r="A4" s="10" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F4" s="5"/>
       <c r="G4" s="5"/>
@@ -920,19 +907,19 @@
     </row>
     <row r="5" spans="1:26" ht="21" customHeight="1">
       <c r="A5" s="10" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F5" s="5"/>
       <c r="G5" s="5"/>
@@ -1042,7 +1029,7 @@
     </row>
     <row r="9" spans="1:26" ht="21" customHeight="1">
       <c r="A9" s="20" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="B9" s="21"/>
       <c r="C9" s="21"/>
@@ -1072,13 +1059,13 @@
     </row>
     <row r="10" spans="1:26" ht="21" customHeight="1">
       <c r="A10" s="22" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B10" s="11"/>
       <c r="C10" s="11"/>
       <c r="D10" s="11"/>
       <c r="E10" s="11" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="F10" s="5"/>
       <c r="G10" s="5"/>
@@ -1104,10 +1091,10 @@
     </row>
     <row r="11" spans="1:26" ht="21" customHeight="1">
       <c r="A11" s="10" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="C11" s="11"/>
       <c r="D11" s="11"/>
@@ -1136,12 +1123,12 @@
     </row>
     <row r="12" spans="1:26" ht="21" customHeight="1">
       <c r="A12" s="10" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B12" s="11"/>
       <c r="C12" s="11"/>
       <c r="D12" s="11" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="E12" s="11"/>
       <c r="F12" s="5"/>
@@ -1168,11 +1155,11 @@
     </row>
     <row r="13" spans="1:26" ht="21" customHeight="1">
       <c r="A13" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B13" s="11"/>
       <c r="C13" s="11" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="11"/>
@@ -1228,7 +1215,7 @@
     </row>
     <row r="15" spans="1:26" ht="21" customHeight="1">
       <c r="A15" s="10" t="s">
-        <v>66</v>
+        <v>45</v>
       </c>
       <c r="B15" s="11"/>
       <c r="C15" s="11"/>
@@ -28885,8 +28872,8 @@
       <c r="Z1" s="4"/>
     </row>
     <row r="2" spans="1:26" ht="21" customHeight="1">
-      <c r="A2" s="4" t="s">
-        <v>8</v>
+      <c r="A2" s="27" t="s">
+        <v>56</v>
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
@@ -28915,8 +28902,8 @@
       <c r="Z2" s="4"/>
     </row>
     <row r="3" spans="1:26" ht="21" customHeight="1">
-      <c r="A3" s="4" t="s">
-        <v>20</v>
+      <c r="A3" s="27" t="s">
+        <v>57</v>
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
@@ -28945,7 +28932,9 @@
       <c r="Z3" s="4"/>
     </row>
     <row r="4" spans="1:26" ht="21" customHeight="1">
-      <c r="A4" s="4"/>
+      <c r="A4" s="27" t="s">
+        <v>58</v>
+      </c>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
       <c r="D4" s="4"/>
@@ -28973,7 +28962,9 @@
       <c r="Z4" s="4"/>
     </row>
     <row r="5" spans="1:26" ht="21" customHeight="1">
-      <c r="A5" s="4"/>
+      <c r="A5" s="27" t="s">
+        <v>59</v>
+      </c>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
@@ -29001,7 +28992,9 @@
       <c r="Z5" s="4"/>
     </row>
     <row r="6" spans="1:26" ht="21" customHeight="1">
-      <c r="A6" s="4"/>
+      <c r="A6" s="27" t="s">
+        <v>60</v>
+      </c>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
       <c r="D6" s="4"/>
@@ -29029,61 +29022,27 @@
       <c r="Z6" s="4"/>
     </row>
     <row r="7" spans="1:26" ht="21" customHeight="1">
-      <c r="A7" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="K7" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="L7" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="M7" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="N7" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="O7" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="P7" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="Q7" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="R7" s="5"/>
-      <c r="S7" s="4"/>
-      <c r="T7" s="4"/>
-      <c r="U7" s="4"/>
+      <c r="A7" s="4"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
+      <c r="L7" s="7"/>
+      <c r="M7" s="7"/>
+      <c r="N7" s="19"/>
+      <c r="O7" s="7"/>
+      <c r="P7" s="7"/>
+      <c r="Q7" s="7"/>
+      <c r="R7" s="7"/>
+      <c r="S7" s="7"/>
+      <c r="T7" s="7"/>
+      <c r="U7" s="7"/>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
       <c r="X7" s="4"/>
@@ -29091,27 +29050,37 @@
       <c r="Z7" s="4"/>
     </row>
     <row r="8" spans="1:26" ht="21" customHeight="1">
-      <c r="A8" s="10"/>
-      <c r="B8" s="11"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11"/>
-      <c r="G8" s="11"/>
-      <c r="H8" s="11"/>
-      <c r="I8" s="11"/>
-      <c r="J8" s="11"/>
-      <c r="K8" s="11"/>
-      <c r="L8" s="11"/>
-      <c r="M8" s="11"/>
-      <c r="N8" s="11"/>
-      <c r="O8" s="11"/>
-      <c r="P8" s="11"/>
-      <c r="Q8" s="23"/>
-      <c r="R8" s="5"/>
-      <c r="S8" s="4"/>
-      <c r="T8" s="4"/>
-      <c r="U8" s="4"/>
+      <c r="A8" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F8" s="19"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="7"/>
+      <c r="J8" s="7"/>
+      <c r="K8" s="7"/>
+      <c r="L8" s="7"/>
+      <c r="M8" s="7"/>
+      <c r="N8" s="19"/>
+      <c r="O8" s="7"/>
+      <c r="P8" s="7"/>
+      <c r="Q8" s="7"/>
+      <c r="R8" s="7"/>
+      <c r="S8" s="7"/>
+      <c r="T8" s="7"/>
+      <c r="U8" s="7"/>
       <c r="V8" s="4"/>
       <c r="W8" s="4"/>
       <c r="X8" s="4"/>
@@ -29119,27 +29088,37 @@
       <c r="Z8" s="4"/>
     </row>
     <row r="9" spans="1:26" ht="21" customHeight="1">
-      <c r="A9" s="10"/>
-      <c r="B9" s="11"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="11"/>
-      <c r="I9" s="11"/>
-      <c r="J9" s="11"/>
-      <c r="K9" s="11"/>
-      <c r="L9" s="11"/>
-      <c r="M9" s="11"/>
-      <c r="N9" s="11"/>
-      <c r="O9" s="11"/>
-      <c r="P9" s="11"/>
-      <c r="Q9" s="23"/>
-      <c r="R9" s="5"/>
-      <c r="S9" s="4"/>
-      <c r="T9" s="4"/>
-      <c r="U9" s="4"/>
+      <c r="A9" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="B9" s="28" t="s">
+        <v>55</v>
+      </c>
+      <c r="C9" s="28" t="s">
+        <v>55</v>
+      </c>
+      <c r="D9" s="28" t="s">
+        <v>55</v>
+      </c>
+      <c r="E9" s="28" t="s">
+        <v>54</v>
+      </c>
+      <c r="F9" s="19"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="7"/>
+      <c r="K9" s="7"/>
+      <c r="L9" s="7"/>
+      <c r="M9" s="7"/>
+      <c r="N9" s="19"/>
+      <c r="O9" s="7"/>
+      <c r="P9" s="7"/>
+      <c r="Q9" s="7"/>
+      <c r="R9" s="7"/>
+      <c r="S9" s="7"/>
+      <c r="T9" s="7"/>
+      <c r="U9" s="7"/>
       <c r="V9" s="4"/>
       <c r="W9" s="4"/>
       <c r="X9" s="4"/>
@@ -29147,27 +29126,37 @@
       <c r="Z9" s="4"/>
     </row>
     <row r="10" spans="1:26" ht="21" customHeight="1">
-      <c r="A10" s="10"/>
-      <c r="B10" s="11"/>
-      <c r="C10" s="11"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="11"/>
-      <c r="G10" s="11"/>
-      <c r="H10" s="11"/>
-      <c r="I10" s="11"/>
-      <c r="J10" s="11"/>
-      <c r="K10" s="11"/>
-      <c r="L10" s="11"/>
-      <c r="M10" s="11"/>
-      <c r="N10" s="11"/>
-      <c r="O10" s="11"/>
-      <c r="P10" s="11"/>
-      <c r="Q10" s="23"/>
-      <c r="R10" s="5"/>
-      <c r="S10" s="4"/>
-      <c r="T10" s="4"/>
-      <c r="U10" s="4"/>
+      <c r="A10" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="B10" s="28" t="s">
+        <v>51</v>
+      </c>
+      <c r="C10" s="28" t="s">
+        <v>52</v>
+      </c>
+      <c r="D10" s="28" t="s">
+        <v>53</v>
+      </c>
+      <c r="E10" s="28" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" s="19"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="7"/>
+      <c r="K10" s="7"/>
+      <c r="L10" s="7"/>
+      <c r="M10" s="7"/>
+      <c r="N10" s="19"/>
+      <c r="O10" s="7"/>
+      <c r="P10" s="7"/>
+      <c r="Q10" s="7"/>
+      <c r="R10" s="7"/>
+      <c r="S10" s="7"/>
+      <c r="T10" s="7"/>
+      <c r="U10" s="7"/>
       <c r="V10" s="4"/>
       <c r="W10" s="4"/>
       <c r="X10" s="4"/>
@@ -29175,29 +29164,27 @@
       <c r="Z10" s="4"/>
     </row>
     <row r="11" spans="1:26" ht="21" customHeight="1">
-      <c r="A11" s="20" t="s">
-        <v>49</v>
-      </c>
+      <c r="A11" s="10"/>
       <c r="B11" s="11"/>
       <c r="C11" s="11"/>
       <c r="D11" s="11"/>
       <c r="E11" s="11"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="11"/>
-      <c r="I11" s="11"/>
-      <c r="J11" s="11"/>
-      <c r="K11" s="10"/>
-      <c r="L11" s="10"/>
-      <c r="M11" s="10"/>
-      <c r="N11" s="10"/>
-      <c r="O11" s="11"/>
-      <c r="P11" s="11"/>
-      <c r="Q11" s="11"/>
-      <c r="R11" s="5"/>
-      <c r="S11" s="4"/>
-      <c r="T11" s="4"/>
-      <c r="U11" s="4"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="7"/>
+      <c r="I11" s="7"/>
+      <c r="J11" s="7"/>
+      <c r="K11" s="7"/>
+      <c r="L11" s="7"/>
+      <c r="M11" s="7"/>
+      <c r="N11" s="19"/>
+      <c r="O11" s="7"/>
+      <c r="P11" s="7"/>
+      <c r="Q11" s="7"/>
+      <c r="R11" s="7"/>
+      <c r="S11" s="7"/>
+      <c r="T11" s="7"/>
+      <c r="U11" s="7"/>
       <c r="V11" s="4"/>
       <c r="W11" s="4"/>
       <c r="X11" s="4"/>
@@ -29205,27 +29192,29 @@
       <c r="Z11" s="4"/>
     </row>
     <row r="12" spans="1:26" ht="21" customHeight="1">
-      <c r="A12" s="10"/>
-      <c r="B12" s="11"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="11"/>
-      <c r="G12" s="11"/>
-      <c r="H12" s="11"/>
-      <c r="I12" s="11"/>
-      <c r="J12" s="11"/>
-      <c r="K12" s="10"/>
-      <c r="L12" s="11"/>
-      <c r="M12" s="10"/>
-      <c r="N12" s="11"/>
-      <c r="O12" s="11"/>
-      <c r="P12" s="11"/>
-      <c r="Q12" s="11"/>
-      <c r="R12" s="5"/>
-      <c r="S12" s="4"/>
-      <c r="T12" s="4"/>
-      <c r="U12" s="4"/>
+      <c r="A12" s="25" t="s">
+        <v>43</v>
+      </c>
+      <c r="B12" s="25"/>
+      <c r="C12" s="25"/>
+      <c r="D12" s="25"/>
+      <c r="E12" s="25"/>
+      <c r="F12" s="19"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="7"/>
+      <c r="J12" s="7"/>
+      <c r="K12" s="7"/>
+      <c r="L12" s="7"/>
+      <c r="M12" s="7"/>
+      <c r="N12" s="19"/>
+      <c r="O12" s="7"/>
+      <c r="P12" s="7"/>
+      <c r="Q12" s="7"/>
+      <c r="R12" s="7"/>
+      <c r="S12" s="7"/>
+      <c r="T12" s="7"/>
+      <c r="U12" s="7"/>
       <c r="V12" s="4"/>
       <c r="W12" s="4"/>
       <c r="X12" s="4"/>
@@ -29233,27 +29222,31 @@
       <c r="Z12" s="4"/>
     </row>
     <row r="13" spans="1:26" ht="21" customHeight="1">
-      <c r="A13" s="10"/>
+      <c r="A13" s="26" t="s">
+        <v>42</v>
+      </c>
       <c r="B13" s="11"/>
       <c r="C13" s="11"/>
       <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="11"/>
-      <c r="H13" s="11"/>
-      <c r="I13" s="11"/>
-      <c r="J13" s="11"/>
-      <c r="K13" s="10"/>
-      <c r="L13" s="11"/>
-      <c r="M13" s="10"/>
-      <c r="N13" s="11"/>
-      <c r="O13" s="11"/>
-      <c r="P13" s="11"/>
-      <c r="Q13" s="11"/>
-      <c r="R13" s="5"/>
-      <c r="S13" s="4"/>
-      <c r="T13" s="4"/>
-      <c r="U13" s="4"/>
+      <c r="E13" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="F13" s="19"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="7"/>
+      <c r="I13" s="7"/>
+      <c r="J13" s="7"/>
+      <c r="K13" s="7"/>
+      <c r="L13" s="7"/>
+      <c r="M13" s="7"/>
+      <c r="N13" s="19"/>
+      <c r="O13" s="7"/>
+      <c r="P13" s="7"/>
+      <c r="Q13" s="7"/>
+      <c r="R13" s="7"/>
+      <c r="S13" s="7"/>
+      <c r="T13" s="7"/>
+      <c r="U13" s="7"/>
       <c r="V13" s="4"/>
       <c r="W13" s="4"/>
       <c r="X13" s="4"/>
@@ -29261,29 +29254,31 @@
       <c r="Z13" s="4"/>
     </row>
     <row r="14" spans="1:26" ht="21" customHeight="1">
-      <c r="A14" s="10" t="s">
-        <v>66</v>
+      <c r="A14" s="26" t="s">
+        <v>36</v>
       </c>
-      <c r="B14" s="11"/>
+      <c r="B14" s="11" t="s">
+        <v>44</v>
+      </c>
       <c r="C14" s="11"/>
       <c r="D14" s="11"/>
       <c r="E14" s="11"/>
-      <c r="F14" s="11"/>
-      <c r="G14" s="11"/>
-      <c r="H14" s="11"/>
-      <c r="I14" s="11"/>
-      <c r="J14" s="11"/>
-      <c r="K14" s="10"/>
-      <c r="L14" s="10"/>
-      <c r="M14" s="10"/>
-      <c r="N14" s="10"/>
-      <c r="O14" s="11"/>
-      <c r="P14" s="11"/>
-      <c r="Q14" s="11"/>
-      <c r="R14" s="5"/>
-      <c r="S14" s="4"/>
-      <c r="T14" s="4"/>
-      <c r="U14" s="4"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="7"/>
+      <c r="K14" s="7"/>
+      <c r="L14" s="7"/>
+      <c r="M14" s="7"/>
+      <c r="N14" s="19"/>
+      <c r="O14" s="7"/>
+      <c r="P14" s="7"/>
+      <c r="Q14" s="7"/>
+      <c r="R14" s="7"/>
+      <c r="S14" s="7"/>
+      <c r="T14" s="7"/>
+      <c r="U14" s="7"/>
       <c r="V14" s="4"/>
       <c r="W14" s="4"/>
       <c r="X14" s="4"/>
@@ -29291,27 +29286,31 @@
       <c r="Z14" s="4"/>
     </row>
     <row r="15" spans="1:26" ht="21" customHeight="1">
-      <c r="A15" s="4"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
-      <c r="I15" s="4"/>
-      <c r="J15" s="4"/>
-      <c r="K15" s="4"/>
-      <c r="L15" s="4"/>
-      <c r="M15" s="4"/>
-      <c r="N15" s="4"/>
-      <c r="O15" s="5"/>
-      <c r="P15" s="5"/>
-      <c r="Q15" s="5"/>
-      <c r="R15" s="5"/>
-      <c r="S15" s="4"/>
-      <c r="T15" s="4"/>
-      <c r="U15" s="4"/>
+      <c r="A15" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B15" s="11"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="E15" s="11"/>
+      <c r="F15" s="19"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="7"/>
+      <c r="I15" s="7"/>
+      <c r="J15" s="7"/>
+      <c r="K15" s="7"/>
+      <c r="L15" s="7"/>
+      <c r="M15" s="7"/>
+      <c r="N15" s="19"/>
+      <c r="O15" s="7"/>
+      <c r="P15" s="7"/>
+      <c r="Q15" s="7"/>
+      <c r="R15" s="7"/>
+      <c r="S15" s="7"/>
+      <c r="T15" s="7"/>
+      <c r="U15" s="7"/>
       <c r="V15" s="4"/>
       <c r="W15" s="4"/>
       <c r="X15" s="4"/>
@@ -29319,27 +29318,31 @@
       <c r="Z15" s="4"/>
     </row>
     <row r="16" spans="1:26" ht="21" customHeight="1">
-      <c r="A16" s="4"/>
-      <c r="B16" s="4"/>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4"/>
-      <c r="I16" s="4"/>
-      <c r="J16" s="4"/>
-      <c r="K16" s="4"/>
-      <c r="L16" s="4"/>
-      <c r="M16" s="4"/>
-      <c r="N16" s="4"/>
-      <c r="O16" s="5"/>
-      <c r="P16" s="5"/>
-      <c r="Q16" s="5"/>
-      <c r="R16" s="5"/>
-      <c r="S16" s="4"/>
-      <c r="T16" s="4"/>
-      <c r="U16" s="4"/>
+      <c r="A16" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B16" s="11"/>
+      <c r="C16" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="7"/>
+      <c r="H16" s="7"/>
+      <c r="I16" s="7"/>
+      <c r="J16" s="7"/>
+      <c r="K16" s="7"/>
+      <c r="L16" s="7"/>
+      <c r="M16" s="7"/>
+      <c r="N16" s="19"/>
+      <c r="O16" s="7"/>
+      <c r="P16" s="7"/>
+      <c r="Q16" s="7"/>
+      <c r="R16" s="7"/>
+      <c r="S16" s="7"/>
+      <c r="T16" s="7"/>
+      <c r="U16" s="7"/>
       <c r="V16" s="4"/>
       <c r="W16" s="4"/>
       <c r="X16" s="4"/>
@@ -29347,27 +29350,27 @@
       <c r="Z16" s="4"/>
     </row>
     <row r="17" spans="1:26" ht="21" customHeight="1">
-      <c r="A17" s="4"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
-      <c r="I17" s="4"/>
-      <c r="J17" s="4"/>
-      <c r="K17" s="4"/>
-      <c r="L17" s="4"/>
-      <c r="M17" s="4"/>
-      <c r="N17" s="4"/>
-      <c r="O17" s="5"/>
-      <c r="P17" s="5"/>
-      <c r="Q17" s="5"/>
-      <c r="R17" s="5"/>
-      <c r="S17" s="4"/>
-      <c r="T17" s="4"/>
-      <c r="U17" s="4"/>
+      <c r="A17" s="26"/>
+      <c r="B17" s="26"/>
+      <c r="C17" s="26"/>
+      <c r="D17" s="26"/>
+      <c r="E17" s="26"/>
+      <c r="F17" s="19"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="7"/>
+      <c r="I17" s="7"/>
+      <c r="J17" s="7"/>
+      <c r="K17" s="7"/>
+      <c r="L17" s="7"/>
+      <c r="M17" s="7"/>
+      <c r="N17" s="19"/>
+      <c r="O17" s="7"/>
+      <c r="P17" s="7"/>
+      <c r="Q17" s="7"/>
+      <c r="R17" s="7"/>
+      <c r="S17" s="7"/>
+      <c r="T17" s="7"/>
+      <c r="U17" s="7"/>
       <c r="V17" s="4"/>
       <c r="W17" s="4"/>
       <c r="X17" s="4"/>
@@ -29375,27 +29378,29 @@
       <c r="Z17" s="4"/>
     </row>
     <row r="18" spans="1:26" ht="21" customHeight="1">
-      <c r="A18" s="4"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
-      <c r="H18" s="4"/>
-      <c r="I18" s="4"/>
-      <c r="J18" s="4"/>
-      <c r="K18" s="4"/>
-      <c r="L18" s="4"/>
-      <c r="M18" s="4"/>
-      <c r="N18" s="4"/>
-      <c r="O18" s="5"/>
-      <c r="P18" s="5"/>
-      <c r="Q18" s="5"/>
-      <c r="R18" s="5"/>
-      <c r="S18" s="4"/>
-      <c r="T18" s="4"/>
-      <c r="U18" s="4"/>
+      <c r="A18" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="B18" s="26"/>
+      <c r="C18" s="26"/>
+      <c r="D18" s="26"/>
+      <c r="E18" s="26"/>
+      <c r="F18" s="19"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="7"/>
+      <c r="I18" s="7"/>
+      <c r="J18" s="7"/>
+      <c r="K18" s="7"/>
+      <c r="L18" s="7"/>
+      <c r="M18" s="7"/>
+      <c r="N18" s="19"/>
+      <c r="O18" s="7"/>
+      <c r="P18" s="7"/>
+      <c r="Q18" s="7"/>
+      <c r="R18" s="7"/>
+      <c r="S18" s="7"/>
+      <c r="T18" s="7"/>
+      <c r="U18" s="7"/>
       <c r="V18" s="4"/>
       <c r="W18" s="4"/>
       <c r="X18" s="4"/>
@@ -29408,22 +29413,22 @@
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
       <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
-      <c r="I19" s="4"/>
-      <c r="J19" s="4"/>
-      <c r="K19" s="4"/>
-      <c r="L19" s="4"/>
-      <c r="M19" s="4"/>
-      <c r="N19" s="4"/>
-      <c r="O19" s="5"/>
-      <c r="P19" s="5"/>
-      <c r="Q19" s="5"/>
-      <c r="R19" s="5"/>
-      <c r="S19" s="4"/>
-      <c r="T19" s="4"/>
-      <c r="U19" s="4"/>
+      <c r="F19" s="19"/>
+      <c r="G19" s="7"/>
+      <c r="H19" s="7"/>
+      <c r="I19" s="7"/>
+      <c r="J19" s="7"/>
+      <c r="K19" s="7"/>
+      <c r="L19" s="7"/>
+      <c r="M19" s="7"/>
+      <c r="N19" s="19"/>
+      <c r="O19" s="7"/>
+      <c r="P19" s="7"/>
+      <c r="Q19" s="7"/>
+      <c r="R19" s="7"/>
+      <c r="S19" s="7"/>
+      <c r="T19" s="7"/>
+      <c r="U19" s="7"/>
       <c r="V19" s="4"/>
       <c r="W19" s="4"/>
       <c r="X19" s="4"/>
@@ -29436,22 +29441,22 @@
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
-      <c r="H20" s="4"/>
-      <c r="I20" s="4"/>
-      <c r="J20" s="4"/>
-      <c r="K20" s="4"/>
-      <c r="L20" s="4"/>
-      <c r="M20" s="4"/>
-      <c r="N20" s="4"/>
-      <c r="O20" s="5"/>
-      <c r="P20" s="5"/>
-      <c r="Q20" s="5"/>
-      <c r="R20" s="5"/>
-      <c r="S20" s="4"/>
-      <c r="T20" s="4"/>
-      <c r="U20" s="4"/>
+      <c r="F20" s="19"/>
+      <c r="G20" s="7"/>
+      <c r="H20" s="7"/>
+      <c r="I20" s="7"/>
+      <c r="J20" s="7"/>
+      <c r="K20" s="7"/>
+      <c r="L20" s="7"/>
+      <c r="M20" s="7"/>
+      <c r="N20" s="19"/>
+      <c r="O20" s="7"/>
+      <c r="P20" s="7"/>
+      <c r="Q20" s="7"/>
+      <c r="R20" s="7"/>
+      <c r="S20" s="7"/>
+      <c r="T20" s="7"/>
+      <c r="U20" s="7"/>
       <c r="V20" s="4"/>
       <c r="W20" s="4"/>
       <c r="X20" s="4"/>
@@ -29464,22 +29469,22 @@
       <c r="C21" s="4"/>
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-      <c r="H21" s="4"/>
-      <c r="I21" s="4"/>
-      <c r="J21" s="4"/>
-      <c r="K21" s="4"/>
-      <c r="L21" s="4"/>
-      <c r="M21" s="4"/>
-      <c r="N21" s="4"/>
-      <c r="O21" s="5"/>
-      <c r="P21" s="5"/>
-      <c r="Q21" s="5"/>
-      <c r="R21" s="5"/>
-      <c r="S21" s="4"/>
-      <c r="T21" s="4"/>
-      <c r="U21" s="4"/>
+      <c r="F21" s="19"/>
+      <c r="G21" s="7"/>
+      <c r="H21" s="7"/>
+      <c r="I21" s="7"/>
+      <c r="J21" s="7"/>
+      <c r="K21" s="7"/>
+      <c r="L21" s="7"/>
+      <c r="M21" s="7"/>
+      <c r="N21" s="19"/>
+      <c r="O21" s="7"/>
+      <c r="P21" s="7"/>
+      <c r="Q21" s="7"/>
+      <c r="R21" s="7"/>
+      <c r="S21" s="7"/>
+      <c r="T21" s="7"/>
+      <c r="U21" s="7"/>
       <c r="V21" s="4"/>
       <c r="W21" s="4"/>
       <c r="X21" s="4"/>
@@ -29492,22 +29497,22 @@
       <c r="C22" s="4"/>
       <c r="D22" s="4"/>
       <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
-      <c r="H22" s="4"/>
-      <c r="I22" s="4"/>
-      <c r="J22" s="4"/>
-      <c r="K22" s="4"/>
-      <c r="L22" s="4"/>
-      <c r="M22" s="4"/>
-      <c r="N22" s="4"/>
-      <c r="O22" s="5"/>
-      <c r="P22" s="5"/>
-      <c r="Q22" s="5"/>
-      <c r="R22" s="5"/>
-      <c r="S22" s="4"/>
-      <c r="T22" s="4"/>
-      <c r="U22" s="4"/>
+      <c r="F22" s="19"/>
+      <c r="G22" s="7"/>
+      <c r="H22" s="7"/>
+      <c r="I22" s="7"/>
+      <c r="J22" s="7"/>
+      <c r="K22" s="7"/>
+      <c r="L22" s="7"/>
+      <c r="M22" s="7"/>
+      <c r="N22" s="19"/>
+      <c r="O22" s="7"/>
+      <c r="P22" s="7"/>
+      <c r="Q22" s="7"/>
+      <c r="R22" s="7"/>
+      <c r="S22" s="7"/>
+      <c r="T22" s="7"/>
+      <c r="U22" s="7"/>
       <c r="V22" s="4"/>
       <c r="W22" s="4"/>
       <c r="X22" s="4"/>
@@ -56920,15 +56925,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="31"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="34"/>
     </row>
     <row r="2" spans="1:8" ht="15.75" customHeight="1">
       <c r="A2" s="6"/>
@@ -56943,46 +56948,46 @@
       <c r="A3" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="32" t="s">
-        <v>9</v>
+      <c r="B3" s="35" t="s">
+        <v>8</v>
       </c>
-      <c r="C3" s="30"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
+      <c r="C3" s="33"/>
+      <c r="D3" s="33"/>
+      <c r="E3" s="33"/>
       <c r="F3" s="12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G3" s="13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A4" s="9" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A4" s="9" t="s">
+      <c r="B4" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="32" t="s">
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33"/>
+      <c r="F4" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="30"/>
-      <c r="F4" s="12" t="s">
+      <c r="G4" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="G4" s="13" t="s">
+    </row>
+    <row r="5" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A5" s="14" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A5" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="B5" s="33"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="31"/>
+      <c r="B5" s="36"/>
+      <c r="C5" s="33"/>
+      <c r="D5" s="33"/>
+      <c r="E5" s="34"/>
       <c r="F5" s="12" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="G5" s="15">
         <v>374961</v>
@@ -56998,42 +57003,42 @@
       <c r="G6" s="7"/>
     </row>
     <row r="7" spans="1:8" ht="27" customHeight="1">
-      <c r="A7" s="34" t="s">
+      <c r="A7" s="37" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="36" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="26" t="s">
+      <c r="D7" s="33"/>
+      <c r="E7" s="34"/>
+      <c r="F7" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="33" t="s">
+      <c r="G7" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="30"/>
-      <c r="E7" s="31"/>
-      <c r="F7" s="26" t="s">
-        <v>30</v>
-      </c>
-      <c r="G7" s="26" t="s">
+      <c r="H7" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="H7" s="28" t="s">
+    </row>
+    <row r="8" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A8" s="30"/>
+      <c r="B8" s="30"/>
+      <c r="C8" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" s="16" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A8" s="27"/>
-      <c r="B8" s="27"/>
-      <c r="C8" s="16" t="s">
+      <c r="E8" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="D8" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="E8" s="16" t="s">
-        <v>36</v>
-      </c>
-      <c r="F8" s="27"/>
-      <c r="G8" s="27"/>
-      <c r="H8" s="27"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
     </row>
     <row r="9" spans="1:8" ht="15.75" customHeight="1">
       <c r="A9" s="17" t="str">
@@ -57041,7 +57046,7 @@
         <v>Rule#1</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C9" s="13">
         <v>1</v>
@@ -57052,14 +57057,14 @@
       <c r="E9" s="13">
         <v>6</v>
       </c>
-      <c r="F9" s="25" t="s">
-        <v>72</v>
+      <c r="F9" s="24" t="s">
+        <v>49</v>
       </c>
-      <c r="G9" s="25" t="s">
-        <v>72</v>
+      <c r="G9" s="24" t="s">
+        <v>49</v>
       </c>
       <c r="H9" s="13" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="15.75" customHeight="1">
@@ -57068,7 +57073,7 @@
         <v>Rule#2</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C10" s="13">
         <v>1</v>
@@ -57079,14 +57084,14 @@
       <c r="E10" s="13">
         <v>1</v>
       </c>
-      <c r="F10" s="25" t="s">
-        <v>71</v>
+      <c r="F10" s="24" t="s">
+        <v>48</v>
       </c>
-      <c r="G10" s="25" t="s">
-        <v>71</v>
+      <c r="G10" s="24" t="s">
+        <v>48</v>
       </c>
       <c r="H10" s="13" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15.75" customHeight="1">
@@ -57095,7 +57100,7 @@
         <v>Rule#3</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C11" s="13">
         <v>1</v>
@@ -57106,14 +57111,14 @@
       <c r="E11" s="13">
         <v>1</v>
       </c>
-      <c r="F11" s="25" t="s">
-        <v>70</v>
+      <c r="F11" s="24" t="s">
+        <v>47</v>
       </c>
-      <c r="G11" s="25" t="s">
-        <v>70</v>
+      <c r="G11" s="24" t="s">
+        <v>47</v>
       </c>
       <c r="H11" s="13" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15.75" customHeight="1">
@@ -57122,7 +57127,7 @@
         <v>Rule#4</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C12" s="13">
         <v>0</v>
@@ -57133,14 +57138,14 @@
       <c r="E12" s="13">
         <v>1</v>
       </c>
-      <c r="F12" s="24" t="s">
-        <v>69</v>
+      <c r="F12" s="23" t="s">
+        <v>46</v>
       </c>
-      <c r="G12" s="24" t="s">
-        <v>69</v>
+      <c r="G12" s="23" t="s">
+        <v>46</v>
       </c>
       <c r="H12" s="13" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="15.75" customHeight="1">
@@ -60208,22 +60213,22 @@
     <col min="1" max="1" width="16.125" customWidth="1"/>
     <col min="2" max="2" width="15.375" customWidth="1"/>
     <col min="3" max="5" width="10.5" customWidth="1"/>
-    <col min="6" max="6" width="17.375" customWidth="1"/>
+    <col min="6" max="6" width="22.25" customWidth="1"/>
     <col min="7" max="7" width="27.875" customWidth="1"/>
     <col min="8" max="8" width="26.5" customWidth="1"/>
     <col min="9" max="26" width="10.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="31"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="34"/>
     </row>
     <row r="2" spans="1:8" ht="15.75" customHeight="1">
       <c r="A2" s="6"/>
@@ -60238,46 +60243,46 @@
       <c r="A3" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="32" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" s="30"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="12" t="s">
+      <c r="B3" s="35" t="s">
         <v>13</v>
       </c>
+      <c r="C3" s="33"/>
+      <c r="D3" s="33"/>
+      <c r="E3" s="33"/>
+      <c r="F3" s="12" t="s">
+        <v>12</v>
+      </c>
       <c r="G3" s="13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A4" s="9" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A4" s="9" t="s">
+      <c r="B4" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="32" t="s">
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33"/>
+      <c r="F4" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="30"/>
-      <c r="F4" s="12" t="s">
+      <c r="G4" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="G4" s="13" t="s">
+    </row>
+    <row r="5" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A5" s="14" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A5" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="B5" s="33"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="31"/>
+      <c r="B5" s="36"/>
+      <c r="C5" s="33"/>
+      <c r="D5" s="33"/>
+      <c r="E5" s="34"/>
       <c r="F5" s="12" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="G5" s="15">
         <v>374961</v>
@@ -60293,212 +60298,163 @@
       <c r="G6" s="7"/>
     </row>
     <row r="7" spans="1:8" ht="55.5" customHeight="1">
-      <c r="A7" s="34" t="s">
+      <c r="A7" s="37" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="36" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="26" t="s">
+      <c r="D7" s="33"/>
+      <c r="E7" s="34"/>
+      <c r="F7" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="33" t="s">
+      <c r="G7" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="30"/>
-      <c r="E7" s="31"/>
-      <c r="F7" s="26" t="s">
-        <v>30</v>
-      </c>
-      <c r="G7" s="26" t="s">
+      <c r="H7" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="H7" s="28" t="s">
+    </row>
+    <row r="8" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A8" s="30"/>
+      <c r="B8" s="30"/>
+      <c r="C8" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" s="16" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A8" s="27"/>
-      <c r="B8" s="27"/>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="27"/>
-      <c r="H8" s="27"/>
+      <c r="E8" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
     </row>
     <row r="9" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A9" s="17"/>
+      <c r="A9" s="17" t="str">
+        <f>("Rule#") &amp; ROW() - 8 &amp; "(EC5, EC1)"</f>
+        <v>Rule#1(EC5, EC1)</v>
+      </c>
       <c r="B9" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" s="13">
+        <v>1</v>
+      </c>
+      <c r="D9" s="13">
+        <v>5</v>
+      </c>
+      <c r="E9" s="13">
+        <v>6</v>
+      </c>
+      <c r="F9" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="G9" s="24"/>
+      <c r="H9" s="13"/>
+    </row>
+    <row r="10" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A10" s="17" t="str">
+        <f>("Rule#") &amp; ROW() - 8 &amp; "(EC5, EC2)"</f>
+        <v>Rule#2(EC5, EC2)</v>
+      </c>
+      <c r="B10" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="13"/>
-      <c r="H9" s="13"/>
-    </row>
-    <row r="10" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A10" s="17"/>
-      <c r="B10" s="13" t="s">
+      <c r="C10" s="13">
+        <v>1</v>
+      </c>
+      <c r="D10" s="13">
+        <v>2</v>
+      </c>
+      <c r="E10" s="13">
+        <v>1</v>
+      </c>
+      <c r="F10" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="G10" s="24"/>
+      <c r="H10" s="13"/>
+    </row>
+    <row r="11" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A11" s="17" t="str">
+        <f>("Rule#") &amp; ROW() - 8 &amp; "(EC5, EC3)"</f>
+        <v>Rule#3(EC5, EC3)</v>
+      </c>
+      <c r="B11" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="13"/>
-      <c r="H10" s="13"/>
-    </row>
-    <row r="11" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A11" s="17"/>
-      <c r="B11" s="13" t="s">
+      <c r="C11" s="13">
+        <v>1</v>
+      </c>
+      <c r="D11" s="13">
+        <v>1</v>
+      </c>
+      <c r="E11" s="13">
+        <v>1</v>
+      </c>
+      <c r="F11" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="G11" s="24"/>
+      <c r="H11" s="13"/>
+    </row>
+    <row r="12" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A12" s="17" t="str">
+        <f>("Rule#") &amp; ROW() - 8 &amp; "(EC4, -)"</f>
+        <v>Rule#4(EC4, -)</v>
+      </c>
+      <c r="B12" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="13"/>
-      <c r="H11" s="13"/>
-    </row>
-    <row r="12" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A12" s="17"/>
-      <c r="B12" s="13" t="s">
-        <v>43</v>
+      <c r="C12" s="13">
+        <v>0</v>
       </c>
-      <c r="C12" s="13"/>
-      <c r="D12" s="13"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13"/>
+      <c r="D12" s="13">
+        <v>1</v>
+      </c>
+      <c r="E12" s="13">
+        <v>1</v>
+      </c>
+      <c r="F12" s="23" t="s">
+        <v>46</v>
+      </c>
+      <c r="G12" s="23"/>
       <c r="H12" s="13"/>
     </row>
     <row r="13" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A13" s="17"/>
-      <c r="B13" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="C13" s="13"/>
-      <c r="D13" s="13"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="13"/>
-      <c r="G13" s="13"/>
-      <c r="H13" s="13"/>
-    </row>
-    <row r="14" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A14" s="17"/>
-      <c r="B14" s="13" t="s">
-        <v>60</v>
-      </c>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="13"/>
-      <c r="H14" s="13"/>
-    </row>
-    <row r="15" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A15" s="17"/>
-      <c r="B15" s="13" t="s">
-        <v>61</v>
-      </c>
-      <c r="C15" s="13"/>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13"/>
-      <c r="H15" s="13"/>
-    </row>
-    <row r="16" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A16" s="17"/>
-      <c r="B16" s="13" t="s">
-        <v>62</v>
-      </c>
-      <c r="C16" s="13"/>
-      <c r="D16" s="13"/>
-      <c r="E16" s="13"/>
-      <c r="F16" s="13"/>
-      <c r="G16" s="13"/>
-      <c r="H16" s="13"/>
-    </row>
-    <row r="17" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A17" s="17"/>
-      <c r="B17" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="C17" s="13"/>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="13"/>
-      <c r="G17" s="13"/>
-      <c r="H17" s="13"/>
-    </row>
-    <row r="18" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A18" s="17"/>
-      <c r="B18" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="13"/>
-      <c r="G18" s="13"/>
-      <c r="H18" s="13"/>
-    </row>
-    <row r="19" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A19" s="17"/>
-      <c r="B19" s="13" t="s">
-        <v>65</v>
-      </c>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="13"/>
-      <c r="F19" s="13"/>
-      <c r="G19" s="13"/>
-      <c r="H19" s="13"/>
-    </row>
-    <row r="20" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A20" s="17"/>
-      <c r="B20" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="13"/>
-      <c r="F20" s="13"/>
-      <c r="G20" s="13"/>
-      <c r="H20" s="13"/>
-    </row>
-    <row r="21" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A21" s="17"/>
-      <c r="B21" s="13" t="s">
-        <v>68</v>
-      </c>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="13"/>
-      <c r="F21" s="13"/>
-      <c r="G21" s="13"/>
-      <c r="H21" s="13"/>
-    </row>
-    <row r="22" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A22" s="6"/>
-      <c r="B22" s="7"/>
-      <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
-      <c r="E22" s="7"/>
-      <c r="F22" s="7"/>
-      <c r="G22" s="7"/>
-    </row>
-    <row r="23" spans="1:8" ht="15.75" customHeight="1"/>
-    <row r="24" spans="1:8" ht="15.75" customHeight="1"/>
-    <row r="25" spans="1:8" ht="15.75" customHeight="1"/>
-    <row r="26" spans="1:8" ht="15.75" customHeight="1"/>
-    <row r="27" spans="1:8" ht="15.75" customHeight="1"/>
-    <row r="28" spans="1:8" ht="15.75" customHeight="1"/>
-    <row r="29" spans="1:8" ht="15.75" customHeight="1"/>
-    <row r="30" spans="1:8" ht="15.75" customHeight="1"/>
-    <row r="31" spans="1:8" ht="15.75" customHeight="1"/>
-    <row r="32" spans="1:8" ht="15.75" customHeight="1"/>
+      <c r="A13" s="6"/>
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+    </row>
+    <row r="14" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="15" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="16" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="17" ht="15.75" customHeight="1"/>
+    <row r="18" ht="15.75" customHeight="1"/>
+    <row r="19" ht="15.75" customHeight="1"/>
+    <row r="20" ht="15.75" customHeight="1"/>
+    <row r="21" ht="15.75" customHeight="1"/>
+    <row r="22" ht="15.75" customHeight="1"/>
+    <row r="23" ht="15.75" customHeight="1"/>
+    <row r="24" ht="15.75" customHeight="1"/>
+    <row r="25" ht="15.75" customHeight="1"/>
+    <row r="26" ht="15.75" customHeight="1"/>
+    <row r="27" ht="15.75" customHeight="1"/>
+    <row r="28" ht="15.75" customHeight="1"/>
+    <row r="29" ht="15.75" customHeight="1"/>
+    <row r="30" ht="15.75" customHeight="1"/>
+    <row r="31" ht="15.75" customHeight="1"/>
+    <row r="32" ht="15.75" customHeight="1"/>
     <row r="33" ht="15.75" customHeight="1"/>
     <row r="34" ht="15.75" customHeight="1"/>
     <row r="35" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
Add lab6_2 for JunitTest and Record results in template_Lab6.xlsx
</commit_message>
<xml_diff>
--- a/Lab06/Test_Cases/template_Lab6.xlsx
+++ b/Lab06/Test_Cases/template_Lab6.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ThirdYearTerm1\Sqa\Lab06\Test_Cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FDD2320-BBDA-4B6C-B5EF-704382D1197A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6519E7BD-013D-46D5-8593-DFB7659CE709}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="63">
   <si>
     <t>Condition</t>
   </si>
@@ -60355,8 +60355,12 @@
       <c r="F9" s="24" t="s">
         <v>49</v>
       </c>
-      <c r="G9" s="24"/>
-      <c r="H9" s="13"/>
+      <c r="G9" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="H9" s="13" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="10" spans="1:8" ht="15.75" customHeight="1">
       <c r="A10" s="17" t="str">
@@ -60378,8 +60382,12 @@
       <c r="F10" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="G10" s="24"/>
-      <c r="H10" s="13"/>
+      <c r="G10" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="H10" s="13" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="11" spans="1:8" ht="15.75" customHeight="1">
       <c r="A11" s="17" t="str">
@@ -60401,8 +60409,12 @@
       <c r="F11" s="24" t="s">
         <v>47</v>
       </c>
-      <c r="G11" s="24"/>
-      <c r="H11" s="13"/>
+      <c r="G11" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="H11" s="13" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="12" spans="1:8" ht="15.75" customHeight="1">
       <c r="A12" s="17" t="str">
@@ -60424,8 +60436,12 @@
       <c r="F12" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="G12" s="23"/>
-      <c r="H12" s="13"/>
+      <c r="G12" s="23" t="s">
+        <v>46</v>
+      </c>
+      <c r="H12" s="13" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="13" spans="1:8" ht="15.75" customHeight="1">
       <c r="A13" s="6"/>

</xml_diff>